<commit_message>
feat: add ZZZGachaLog template and update Genshin template
fix misalignment
</commit_message>
<xml_diff>
--- a/Starward.Assets/Assets/Template/GachaLog.xlsx
+++ b/Starward.Assets/Assets/Template/GachaLog.xlsx
@@ -1,143 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4E6096-2242-4615-A821-6E93C03109D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{56A29EF9-91E6-449E-BE86-3AB4E7A0A097}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gacha Log" sheetId="1" r:id="rId1"/>
+    <sheet name="Gacha Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gacha Log'!$A$1:$I$2</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
-  <si>
-    <t>gacha_type</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>item_type</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>rank_type</t>
-  </si>
-  <si>
-    <t>time</t>
-  </si>
-  <si>
-    <t>uid</t>
-  </si>
-  <si>
-    <t>{{list.Uid}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Time}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Name}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.ItemType}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.RankType}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.GachaType}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>pity</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Index}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Pity}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>index</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.IdText}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="164" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FF0070C0"/>
       <sz val="11"/>
-      <color rgb="FF0070C0"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FF808080"/>
       <sz val="11"/>
-      <color rgb="FF808080"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -153,18 +75,25 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -204,21 +133,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF808080"/>
-      <color rgb="FFA256E1"/>
-      <color rgb="FFBD6932"/>
-    </mruColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -518,102 +433,141 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1EFA00-53F9-410A-BA16-B5F49C209269}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="26.4140625" customWidth="1"/>
-    <col min="3" max="3" width="22.58203125" customWidth="1"/>
-    <col min="4" max="4" width="15.25" customWidth="1"/>
-    <col min="5" max="5" width="12.75" customWidth="1"/>
-    <col min="6" max="6" width="10.58203125" customWidth="1"/>
-    <col min="7" max="7" width="22.58203125" customWidth="1"/>
-    <col min="8" max="9" width="9.75" customWidth="1"/>
+    <col width="15" customWidth="1" style="3" min="1" max="1"/>
+    <col width="26.4140625" customWidth="1" style="3" min="2" max="2"/>
+    <col width="22.58203125" customWidth="1" style="3" min="3" max="3"/>
+    <col width="15.25" customWidth="1" style="3" min="4" max="4"/>
+    <col width="12.75" customWidth="1" style="3" min="5" max="5"/>
+    <col width="10.58203125" customWidth="1" style="3" min="6" max="6"/>
+    <col width="22.58203125" customWidth="1" style="3" min="7" max="7"/>
+    <col width="9.75" customWidth="1" style="3" min="8" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>13</v>
+    <row r="1" ht="16.5" customHeight="1" s="3">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>uid</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>item_type</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>rank_type</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>gacha_type</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>pity</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>15</v>
+    <row r="2" ht="16.5" customHeight="1" s="3">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Uid}}</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.IdText}}</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Time}}</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Name}}</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.ItemType}}</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.RankType}}</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.GachaType}}</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Index}}</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Pity}}</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I2" xr:uid="{6A1EFA00-53F9-410A-BA16-B5F49C209269}"/>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="A1:I1048576">
-    <cfRule type="expression" dxfId="5" priority="49">
-      <formula>$F1="5"</formula>
+  <autoFilter ref="A1:I2"/>
+  <conditionalFormatting sqref="A2:I1048576">
+    <cfRule type="expression" priority="49" dxfId="4">
+      <formula>$F2="5"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="50">
-      <formula>$F1=5</formula>
+    <cfRule type="expression" priority="50" dxfId="4">
+      <formula>$F2=5</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="51">
-      <formula>$F1="4"</formula>
+    <cfRule type="expression" priority="51" dxfId="2">
+      <formula>$F2="4"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="52">
-      <formula>$F1=4</formula>
+    <cfRule type="expression" priority="52" dxfId="2">
+      <formula>$F2=4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="53">
-      <formula>$F1="3"</formula>
+    <cfRule type="expression" priority="53" dxfId="0">
+      <formula>$F2="3"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="54">
-      <formula>$F1=3</formula>
+    <cfRule type="expression" priority="54" dxfId="0">
+      <formula>$F2=3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add ZZZGachaLog template and update Genshin template (#1871)
fix misalignment
</commit_message>
<xml_diff>
--- a/Starward.Assets/Assets/Template/GachaLog.xlsx
+++ b/Starward.Assets/Assets/Template/GachaLog.xlsx
@@ -1,143 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4E6096-2242-4615-A821-6E93C03109D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{56A29EF9-91E6-449E-BE86-3AB4E7A0A097}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gacha Log" sheetId="1" r:id="rId1"/>
+    <sheet name="Gacha Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gacha Log'!$A$1:$I$2</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
-  <si>
-    <t>gacha_type</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>item_type</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>rank_type</t>
-  </si>
-  <si>
-    <t>time</t>
-  </si>
-  <si>
-    <t>uid</t>
-  </si>
-  <si>
-    <t>{{list.Uid}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Time}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Name}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.ItemType}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.RankType}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.GachaType}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>pity</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Index}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.Pity}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>index</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{list.IdText}}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="164" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FF0070C0"/>
       <sz val="11"/>
-      <color rgb="FF0070C0"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="等线"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="9"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FF808080"/>
       <sz val="11"/>
-      <color rgb="FF808080"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -153,18 +75,25 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -204,21 +133,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF808080"/>
-      <color rgb="FFA256E1"/>
-      <color rgb="FFBD6932"/>
-    </mruColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -518,102 +433,141 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1EFA00-53F9-410A-BA16-B5F49C209269}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="26.4140625" customWidth="1"/>
-    <col min="3" max="3" width="22.58203125" customWidth="1"/>
-    <col min="4" max="4" width="15.25" customWidth="1"/>
-    <col min="5" max="5" width="12.75" customWidth="1"/>
-    <col min="6" max="6" width="10.58203125" customWidth="1"/>
-    <col min="7" max="7" width="22.58203125" customWidth="1"/>
-    <col min="8" max="9" width="9.75" customWidth="1"/>
+    <col width="15" customWidth="1" style="3" min="1" max="1"/>
+    <col width="26.4140625" customWidth="1" style="3" min="2" max="2"/>
+    <col width="22.58203125" customWidth="1" style="3" min="3" max="3"/>
+    <col width="15.25" customWidth="1" style="3" min="4" max="4"/>
+    <col width="12.75" customWidth="1" style="3" min="5" max="5"/>
+    <col width="10.58203125" customWidth="1" style="3" min="6" max="6"/>
+    <col width="22.58203125" customWidth="1" style="3" min="7" max="7"/>
+    <col width="9.75" customWidth="1" style="3" min="8" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>13</v>
+    <row r="1" ht="16.5" customHeight="1" s="3">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>uid</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>item_type</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>rank_type</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>gacha_type</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>pity</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>15</v>
+    <row r="2" ht="16.5" customHeight="1" s="3">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Uid}}</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.IdText}}</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Time}}</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Name}}</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.ItemType}}</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.RankType}}</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.GachaType}}</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Index}}</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>{{list.Pity}}</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I2" xr:uid="{6A1EFA00-53F9-410A-BA16-B5F49C209269}"/>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="A1:I1048576">
-    <cfRule type="expression" dxfId="5" priority="49">
-      <formula>$F1="5"</formula>
+  <autoFilter ref="A1:I2"/>
+  <conditionalFormatting sqref="A2:I1048576">
+    <cfRule type="expression" priority="49" dxfId="4">
+      <formula>$F2="5"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="50">
-      <formula>$F1=5</formula>
+    <cfRule type="expression" priority="50" dxfId="4">
+      <formula>$F2=5</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="51">
-      <formula>$F1="4"</formula>
+    <cfRule type="expression" priority="51" dxfId="2">
+      <formula>$F2="4"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="52">
-      <formula>$F1=4</formula>
+    <cfRule type="expression" priority="52" dxfId="2">
+      <formula>$F2=4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="53">
-      <formula>$F1="3"</formula>
+    <cfRule type="expression" priority="53" dxfId="0">
+      <formula>$F2="3"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="54">
-      <formula>$F1=3</formula>
+    <cfRule type="expression" priority="54" dxfId="0">
+      <formula>$F2=3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>